<commit_message>
Fill the permit tracker with the uploaded firm list.
The workbook now has all 67 firms from the Firmalar list, with blank license and opinion columns that can be set from a yes/no dropdown.

Co-authored-by: iremalisan <iremalisan@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/cevre-izin-takip.xlsx
+++ b/cevre-izin-takip.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Açıklama" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Çevre izin takibi'!$A$1:$C$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Çevre izin takibi'!$A$1:$D$100</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Çevre izin takibi'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -102,10 +102,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -510,251 +510,1036 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:D100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="88" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="92" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Sıra</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Firma adı</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Çevre izin lisansı var mı?</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Çevre izin görüşü var mı?</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>MEDCEM MADENCİLİK VE YAPI MALZEMELERİ SAN.TİC.A.Ş. SİLİFKE ŞUBESİ</t>
-        </is>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="n"/>
-    </row>
-    <row r="3" ht="36" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>MEDCEM MADENCİLİK VEYAPI MALZEMELERİSAN.TİC.A.Ş.</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n"/>
-    </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>RAMAZAN KOÇYİĞİT METAL HURDACILIK PLASTİK AKARYAKIT İNŞAAT SANAYİ VE TİCARET LİMİTED ŞİRKETİ-MERSİN ŞUBESİ</t>
-        </is>
+          <t>Başhan Agro Gıda Sanayi ve Ticaret Anonim Şirketi</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Başhan Agro Gıda Sanayi ve Ticaret A. Ş. Entegre Mersin Şubesi</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n"/>
-    </row>
-    <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>TURYAM GERİ KAZANIM ATIKTAN TÜRETİLMİŞ YAKIT DEPOLAMA LOJİSTİK PETROL ÜRÜNLERİ İNŞAAT MEDİKAL TURİZM SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n"/>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>ÇİMSA ÇİMENTO SANAYİ VE TİCARET ANONİM ŞİRKETİ</t>
-        </is>
+          <t>Organivo Via Gübre İmalat İth. İhr. San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>DEMKOÇ Metal İmalat San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n"/>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>OYAK ÇİMENTO FABRİKALARI A.Ş. ADANA ÇİMENTO ŞUBESİ</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n"/>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>YILDIRIM ATIK VE MADENİ YAĞ GERİ DÖNÜŞÜM ATIKTAN TÜRETİLMİŞ YAKIT HAZIRLAMA NAKLİYE PAZARLAMA SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
-        </is>
+          <t>Şah Oil Madeni Yağ Geri Kaz. Nak. İnş. San. ve Tic. A.Ş.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>YILPACK Ambalaj San. ve Tic. A.Ş. Adana Şubesi</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="n"/>
-    </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>İBC GERİ DÖNÜŞÜM HURDA NAKLİYAT DIŞ TİCARET SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n"/>
-    </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>İSKENDERUN ENERJİ ÜRETİM TİC.A.Ş.</t>
-        </is>
+          <t>Sabuncular Soğuk Hava Deposu Kömürcülük Gıda Tarım Ürünleri Nak. İnş. Taahhüt Ambalaj Sanayi ve Ticaret Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Uyarlar İnş. Mak. Çelik. Konst. Tes. İml. Mont. Turz. San. Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Evet</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="n"/>
-    </row>
-    <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-    </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-    </row>
-    <row r="13" ht="36" customHeight="1">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
-    </row>
-    <row r="14" ht="36" customHeight="1">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-    </row>
-    <row r="15" ht="36" customHeight="1">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-    </row>
-    <row r="16" ht="36" customHeight="1">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-    </row>
-    <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
-    </row>
-    <row r="18" ht="36" customHeight="1">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="n"/>
-    </row>
-    <row r="19" ht="36" customHeight="1">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-    </row>
-    <row r="20" ht="36" customHeight="1">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n"/>
-    </row>
-    <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="2" t="n"/>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
-    </row>
-    <row r="22" ht="36" customHeight="1">
-      <c r="A22" s="2" t="n"/>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-    </row>
-    <row r="23" ht="36" customHeight="1">
-      <c r="A23" s="2" t="n"/>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-    </row>
-    <row r="24" ht="36" customHeight="1">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="3" t="n"/>
-    </row>
-    <row r="25" ht="36" customHeight="1">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-    </row>
-    <row r="26" ht="36" customHeight="1">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
-    </row>
-    <row r="27" ht="36" customHeight="1">
-      <c r="A27" s="2" t="n"/>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="n"/>
-    </row>
-    <row r="28" ht="36" customHeight="1">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="3" t="n"/>
-      <c r="C28" s="3" t="n"/>
-    </row>
-    <row r="29" ht="36" customHeight="1">
-      <c r="A29" s="2" t="n"/>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-    </row>
-    <row r="30" ht="36" customHeight="1">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="3" t="n"/>
-      <c r="C30" s="3" t="n"/>
+          <t>ÖZ-KA Tarım Ürünleri İth. İhr. ve Tic. Ltd. Şti. Adana Sanayi Şubesi</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Tıtan2 Ic İçtaş İnşaat Anonim Şirketi</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Emrenes Orman Ürünleri Sanayi ve Ticaret Ltd. Şti. (Toplama Ayırma)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Armada Duvar Kâğıtları Anonim Şirketi</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Kılıçoğlu Hurdacılık -OKAN KILIÇ (Toplama Ayırma)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>AMİBLU Turkey Boru Sanayi ve Ticaret A.Ş.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>CVD MADENCİLİK LTD. ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Kemaş Kimya Endüstri Merkezi Sanayi ve Ticaret A.Ş.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>İlkesilis Madencilik Sanayi ve Ticaret Limited Şirketi</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>ATS Altuntaş Geri Kazanım Atık Depolama San. ve Tic. Ltd. Şti. (Toplama Ayırma)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>OZCAN Mühendislik Çelik İmalat İnşaat San. ve Tic. Ltd. Şti. Silifke Şubesi</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Marde Hotel-Uçan Turizm Seyahat İnş. Tic. ve San. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Soyerler Gıda Tarım Ürünleri Maden Suları İnşaat İthalat İhracat Sanayi Ve Ticaret Limited Şirketi</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>MGD Gıda Dış Ticaret Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Çukurova Çelik Hasır Demir Metal İnş. Alüminyum İth. İhr. San. ve Tic. A.Ş.</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>TEKNOPARS Makine İmalat San. Tic. A.Ş.</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>MESKİM Gıda İth. İhr. San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Kervan İnşaat-Barbarossa Oteli</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Salt Cam San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Salt Cam San. ve Tic. Ltd. Şti. Nacarlı Osb Temper 2 Şubesi</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+    </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Berrak Doğal Kaynak Suları ve Tic. A.Ş. Tarsus Berrak Su</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>NSS Mühendislik Danışmanlık San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+    </row>
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>CANPACK Tarım Turz. İnş. San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+    </row>
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Başaranlar Plastik İml. San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+    </row>
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>ÖNER Tarım Gıda İth. İhr. A.Ş.</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+    </row>
+    <row r="35" ht="32" customHeight="1">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>ÖNER Seperatör Sanayi Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Abdulkadir ÖZTÜRK-ASLAN TEL</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+    </row>
+    <row r="37" ht="32" customHeight="1">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Akdeniz Prekast Beton Yapı İnşaat Taahhüt Limited Şirketi</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+    </row>
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Merlas Oto Lastik Endüstri San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+    </row>
+    <row r="39" ht="32" customHeight="1">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Merkap Oto Lastik Endüstri San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+    </row>
+    <row r="40" ht="32" customHeight="1">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>TATŞEN Pazarlama Gıda Sanayi ve Ticaret Limited Şirketi</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+    </row>
+    <row r="41" ht="32" customHeight="1">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>ORGÜB Organik Gübre Kükürt Tarım Ürünleri Makina Maden San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+    </row>
+    <row r="42" ht="32" customHeight="1">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>GOLDENNUTS Gıda İthalat İhracat Sanayi ve Ticaret Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+    </row>
+    <row r="43" ht="32" customHeight="1">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Karanlar Petrol Ürünleri İnş. Nak. Tar. Tur. San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+    </row>
+    <row r="44" ht="32" customHeight="1">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Kılıç Tarım Gıda Harf. Pet. Tur. San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+    </row>
+    <row r="45" ht="32" customHeight="1">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Kılıçhedef Tarımsal Ürt. Paz. Tur. Tic. ve San. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+    </row>
+    <row r="46" ht="32" customHeight="1">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>SCA Metal İnşaat Taahhüt Yalıtım İzolasyon San. ve Tic. A.Ş.</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+    </row>
+    <row r="47" ht="32" customHeight="1">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>SB Lotus Turizm İnş. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+    </row>
+    <row r="48" ht="32" customHeight="1">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Coşkun Otomotiv San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+    </row>
+    <row r="49" ht="32" customHeight="1">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Lion Plastik Nakliye Gıda Orman Ürünleri San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" s="2" t="n"/>
+    </row>
+    <row r="50" ht="32" customHeight="1">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>ERAY PARILTI - ERPA PLASTİK</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+    </row>
+    <row r="51" ht="32" customHeight="1">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>İnci Bulgur Sanayi ve Ticaret A.Ş. Mersin Kazanlı Şubesi</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="2" t="n"/>
+    </row>
+    <row r="52" ht="32" customHeight="1">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Kuzgun İmalat Otomotiv İth. İhr. San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="n"/>
+      <c r="D52" s="2" t="n"/>
+    </row>
+    <row r="53" ht="32" customHeight="1">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>ES ŞİMŞEK Plastik Hurdacılık San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="n"/>
+      <c r="D53" s="2" t="n"/>
+    </row>
+    <row r="54" ht="32" customHeight="1">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Cengiz UÇAR-UÇAR Otomotiv</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" s="2" t="n"/>
+    </row>
+    <row r="55" ht="32" customHeight="1">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Trento Lojistik ve Kiralama Operasyonları A.Ş. Mersin Şubesi</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="n"/>
+      <c r="D55" s="2" t="n"/>
+    </row>
+    <row r="56" ht="32" customHeight="1">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>CMA Makina İmalat İth. İhr. San. ve Tic. Ltd. Şti. Sarıçam Şubesi</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
+    </row>
+    <row r="57" ht="32" customHeight="1">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Master Packing Tarım Ürünleri Paketleme İhracat Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+    </row>
+    <row r="58" ht="32" customHeight="1">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Efecan Badem Aromatik Bitkiler Yağlar Gıda Orman Ür. San. ve Tic. A.Ş.</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="n"/>
+      <c r="D58" s="2" t="n"/>
+    </row>
+    <row r="59" ht="32" customHeight="1">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Efecan Badem Aromatik Bitkiler Yağlar Gıda Orman Ürünleri San. ve Tic. A.Ş. Tarsus OSB Şubesi</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="n"/>
+      <c r="D59" s="2" t="n"/>
+    </row>
+    <row r="60" ht="32" customHeight="1">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Aktoğ Uluslararası Nakliyat Otomotiv ve Petrol Ürünleri Sanayi Ticaret Limitd Şirketi</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="n"/>
+      <c r="D60" s="2" t="n"/>
+    </row>
+    <row r="61" ht="32" customHeight="1">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Ünal PIÇAKÇI</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="n"/>
+      <c r="D61" s="2" t="n"/>
+    </row>
+    <row r="62" ht="32" customHeight="1">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Arif KOÇYİĞİT</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="n"/>
+      <c r="D62" s="2" t="n"/>
+    </row>
+    <row r="63" ht="32" customHeight="1">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Özden ÇOĞUL</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="n"/>
+      <c r="D63" s="2" t="n"/>
+    </row>
+    <row r="64" ht="32" customHeight="1">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Osman ÇOĞUL-İkizler Metal Hurda</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="n"/>
+      <c r="D64" s="2" t="n"/>
+    </row>
+    <row r="65" ht="32" customHeight="1">
+      <c r="A65" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Hakan KILIÇ</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="n"/>
+      <c r="D65" s="2" t="n"/>
+    </row>
+    <row r="66" ht="32" customHeight="1">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Arı Hurdacılık Demir Çelik İnş. M. Nak. San. ve Tic. Ltd. Şti.</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="n"/>
+      <c r="D66" s="2" t="n"/>
+    </row>
+    <row r="67" ht="32" customHeight="1">
+      <c r="A67" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Gündüz Mey-Pak Gıda İnş. Taş. Oto. Pet. Ürün. Tur. Tic. Ltd. Şti. Akdeniz Şubesi</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="n"/>
+      <c r="D67" s="2" t="n"/>
+    </row>
+    <row r="68" ht="32" customHeight="1">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>DASBLUE KİMYA SANAYİ TİCARET LİMİTED ŞİRKETİ</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="n"/>
+      <c r="D68" s="2" t="n"/>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="2" t="n"/>
+      <c r="B69" s="3" t="n"/>
+      <c r="C69" s="2" t="n"/>
+      <c r="D69" s="2" t="n"/>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="2" t="n"/>
+      <c r="B70" s="3" t="n"/>
+      <c r="C70" s="2" t="n"/>
+      <c r="D70" s="2" t="n"/>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="2" t="n"/>
+      <c r="B71" s="3" t="n"/>
+      <c r="C71" s="2" t="n"/>
+      <c r="D71" s="2" t="n"/>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="2" t="n"/>
+      <c r="B72" s="3" t="n"/>
+      <c r="C72" s="2" t="n"/>
+      <c r="D72" s="2" t="n"/>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="2" t="n"/>
+      <c r="B73" s="3" t="n"/>
+      <c r="C73" s="2" t="n"/>
+      <c r="D73" s="2" t="n"/>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="2" t="n"/>
+      <c r="B74" s="3" t="n"/>
+      <c r="C74" s="2" t="n"/>
+      <c r="D74" s="2" t="n"/>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="2" t="n"/>
+      <c r="B75" s="3" t="n"/>
+      <c r="C75" s="2" t="n"/>
+      <c r="D75" s="2" t="n"/>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="2" t="n"/>
+      <c r="B76" s="3" t="n"/>
+      <c r="C76" s="2" t="n"/>
+      <c r="D76" s="2" t="n"/>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="2" t="n"/>
+      <c r="B77" s="3" t="n"/>
+      <c r="C77" s="2" t="n"/>
+      <c r="D77" s="2" t="n"/>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="2" t="n"/>
+      <c r="B78" s="3" t="n"/>
+      <c r="C78" s="2" t="n"/>
+      <c r="D78" s="2" t="n"/>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="2" t="n"/>
+      <c r="B79" s="3" t="n"/>
+      <c r="C79" s="2" t="n"/>
+      <c r="D79" s="2" t="n"/>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="2" t="n"/>
+      <c r="B80" s="3" t="n"/>
+      <c r="C80" s="2" t="n"/>
+      <c r="D80" s="2" t="n"/>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="2" t="n"/>
+      <c r="B81" s="3" t="n"/>
+      <c r="C81" s="2" t="n"/>
+      <c r="D81" s="2" t="n"/>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="2" t="n"/>
+      <c r="B82" s="3" t="n"/>
+      <c r="C82" s="2" t="n"/>
+      <c r="D82" s="2" t="n"/>
+    </row>
+    <row r="83" ht="22" customHeight="1">
+      <c r="A83" s="2" t="n"/>
+      <c r="B83" s="3" t="n"/>
+      <c r="C83" s="2" t="n"/>
+      <c r="D83" s="2" t="n"/>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="2" t="n"/>
+      <c r="B84" s="3" t="n"/>
+      <c r="C84" s="2" t="n"/>
+      <c r="D84" s="2" t="n"/>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="2" t="n"/>
+      <c r="B85" s="3" t="n"/>
+      <c r="C85" s="2" t="n"/>
+      <c r="D85" s="2" t="n"/>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="2" t="n"/>
+      <c r="B86" s="3" t="n"/>
+      <c r="C86" s="2" t="n"/>
+      <c r="D86" s="2" t="n"/>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="2" t="n"/>
+      <c r="B87" s="3" t="n"/>
+      <c r="C87" s="2" t="n"/>
+      <c r="D87" s="2" t="n"/>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="2" t="n"/>
+      <c r="B88" s="3" t="n"/>
+      <c r="C88" s="2" t="n"/>
+      <c r="D88" s="2" t="n"/>
+    </row>
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="2" t="n"/>
+      <c r="B89" s="3" t="n"/>
+      <c r="C89" s="2" t="n"/>
+      <c r="D89" s="2" t="n"/>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="2" t="n"/>
+      <c r="B90" s="3" t="n"/>
+      <c r="C90" s="2" t="n"/>
+      <c r="D90" s="2" t="n"/>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="2" t="n"/>
+      <c r="B91" s="3" t="n"/>
+      <c r="C91" s="2" t="n"/>
+      <c r="D91" s="2" t="n"/>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="A92" s="2" t="n"/>
+      <c r="B92" s="3" t="n"/>
+      <c r="C92" s="2" t="n"/>
+      <c r="D92" s="2" t="n"/>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="2" t="n"/>
+      <c r="B93" s="3" t="n"/>
+      <c r="C93" s="2" t="n"/>
+      <c r="D93" s="2" t="n"/>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="2" t="n"/>
+      <c r="B94" s="3" t="n"/>
+      <c r="C94" s="2" t="n"/>
+      <c r="D94" s="2" t="n"/>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="2" t="n"/>
+      <c r="B95" s="3" t="n"/>
+      <c r="C95" s="2" t="n"/>
+      <c r="D95" s="2" t="n"/>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="2" t="n"/>
+      <c r="B96" s="3" t="n"/>
+      <c r="C96" s="2" t="n"/>
+      <c r="D96" s="2" t="n"/>
+    </row>
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="2" t="n"/>
+      <c r="B97" s="3" t="n"/>
+      <c r="C97" s="2" t="n"/>
+      <c r="D97" s="2" t="n"/>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="2" t="n"/>
+      <c r="B98" s="3" t="n"/>
+      <c r="C98" s="2" t="n"/>
+      <c r="D98" s="2" t="n"/>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="2" t="n"/>
+      <c r="B99" s="3" t="n"/>
+      <c r="C99" s="2" t="n"/>
+      <c r="D99" s="2" t="n"/>
+    </row>
+    <row r="100" ht="22" customHeight="1">
+      <c r="A100" s="2" t="n"/>
+      <c r="B100" s="3" t="n"/>
+      <c r="C100" s="2" t="n"/>
+      <c r="D100" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C30"/>
-  <conditionalFormatting sqref="B2:C30">
+  <autoFilter ref="A1:D100"/>
+  <conditionalFormatting sqref="C2:D100">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Evet"</formula>
     </cfRule>
@@ -763,11 +1548,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="B2:C30" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz seçim" error="Hücreye Evet veya Hayır yazın ya da listeden seçin." promptTitle="Seçim" prompt="Evet veya Hayır seçebilirsiniz. Boş bırakmak da mümkündür." type="list">
+    <dataValidation sqref="C2:D100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz seçim" error="Hücreye Evet veya Hayır yazın ya da listeden seçin." promptTitle="Seçim" prompt="Evet veya Hayır seçebilirsiniz. Boş bırakmak da mümkündür." type="list">
       <formula1>"Evet,Hayır"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageMargins left="0.45" right="0.45" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LÇevre izin lisansı ve görüş takibi</oddHeader>
@@ -786,7 +1571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -800,87 +1585,51 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="48" customHeight="1">
+    <row r="3" ht="42" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Ne işe yarar</t>
+          <t>Liste</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Firma adının yanında iki soru vardır: çevre izin lisansı var mı, çevre izin görüşü var mı. Hücreye tıklayıp listeden Evet veya Hayır seçebilir, firma adını değiştirebilir, boş satıra yeni firma yazabilirsiniz.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="48" customHeight="1">
+          <t>67 firma, gönderilen Firmalar listesindeki sıra ile yazıldı. Satır numarası dosyadaki firma sayısıdır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
+          <t>Sütunlar</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Firma adının yanında iki soru vardır: çevre izin lisansı var mı, çevre izin görüşü var mı. Bu iki bilgi kaynak listede yoktu; hücreler boş bırakıldı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
           <t>Nasıl değiştirilir</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>B ve C sütunlarında açılır liste vardır. Liste dışında bir değer yazılırsa Excel uyarı verir. İstediğiniz satırı silebilir veya 30. satıra kadar yeni firma ekleyebilirsiniz.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Başlangıç listesi</t>
-        </is>
-      </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>İlk 9 firma, 6 Ekim 2026 tarihli e-izin belge aramasından alınmıştır. Kaynak: https://eizin.cevre.gov.tr/Rapor/BelgeArama.aspx — belge tipi Çevre İzin ve Lisans Belgesi; Mersin ve Adana; atık kodları 150110 ve 150202 birlikte.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="48" customHeight="1">
+          <t>C ve D sütunlarında açılır liste vardır. Evet veya Hayır seçin, firma adını değiştirin, 100. satıra kadar yeni firma yazın.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Lisans sütunu</t>
+          <t>Renk</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Bu firmalar o sorguda Çevre İzin ve Lisans Belgesi ile göründüğü için çevre izin lisansı Evet olarak işaretlendi. Belge süresi dolmuş veya yeniden düzenlenmiş olabilir; resmi kayıttan kontrol edin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Görüş sütunu</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Aynı sorguda çevre izin görüşü ayrı bir sonuç değildir. Bu yüzden görüş hücreleri boş bırakıldı. Elinizdeki görüş yazısına göre Evet veya Hayır seçin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>İl ayrımı</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>İlk 5 firma Mersin sorgusundan, sonraki 4 firma Adana sorgusundandır.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>İndirme</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Dosyayı Excel veya uyumlu bir hesap tablosu programında açın. Değişiklikler dosyanın içinde kalır; kaydedince güncel tablo sizde durur.</t>
+          <t>Evet yeşil, Hayır kırmızı görünür. Seçimi değiştirince renk de güncellenir.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Treat environmental opinion as unnecessary when a license exists.
A firm with an environmental permit license no longer needs an opinion: the opinion cell accepts Gerekmez and the explanation sheet records the rule.

Co-authored-by: iremalisan <iremalisan@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/cevre-izin-takip.xlsx
+++ b/cevre-izin-takip.xlsx
@@ -121,7 +121,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
     <dxf>
       <font>
         <name val="Calibri"/>
@@ -145,6 +145,20 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00F8D0D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="001F4E79"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D6E3F0"/>
+          <bgColor rgb="00D6E3F0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1546,10 +1560,16 @@
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
       <formula>"Hayır"</formula>
     </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Gerekmez"</formula>
+    </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation sqref="C2:D100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz seçim" error="Hücreye Evet veya Hayır yazın ya da listeden seçin." promptTitle="Seçim" prompt="Evet veya Hayır seçebilirsiniz. Boş bırakmak da mümkündür." type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="C2:C100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz seçim" error="Hücreye Evet veya Hayır yazın ya da listeden seçin." promptTitle="Lisans" prompt="Evet veya Hayır seçebilirsiniz. Lisans Evet ise görüş gerekmez." type="list">
       <formula1>"Evet,Hayır"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz seçim" error="Hücreye Evet, Hayır veya Gerekmez yazın ya da listeden seçin." promptTitle="Görüş" prompt="Lisans yoksa Evet veya Hayır seçin. Lisans varsa Gerekmez yazın." type="list">
+      <formula1>"Evet,Hayır,Gerekmez"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.45" right="0.45" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
@@ -1571,7 +1591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1617,7 +1637,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>C ve D sütunlarında açılır liste vardır. Evet veya Hayır seçin, firma adını değiştirin, 100. satıra kadar yeni firma yazın.</t>
+          <t>C sütununda Evet veya Hayır seçin. Lisans Evet ise görüş gerekmez; D sütununa Gerekmez yazın. Lisans yoksa D sütununda Evet veya Hayır seçin.</t>
         </is>
       </c>
     </row>
@@ -1629,7 +1649,19 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Evet yeşil, Hayır kırmızı görünür. Seçimi değiştirince renk de güncellenir.</t>
+          <t>Evet yeşil, Hayır kırmızı, Gerekmez mavi görünür. Seçimi değiştirince renk de güncellenir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Kural</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Çevre izin lisansı varsa çevre izin görüşü aranmaz. Lisans hücresi Evet olunca görüş hücresine Gerekmez yazılır.</t>
         </is>
       </c>
     </row>

</xml_diff>